<commit_message>
Initial commit by DevOps Concierge Agent
</commit_message>
<xml_diff>
--- a/api_key_metrics.xlsx
+++ b/api_key_metrics.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K546"/>
+  <dimension ref="A1:K558"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -29482,6 +29482,642 @@
         </is>
       </c>
     </row>
+    <row r="547" ht="20" customHeight="1">
+      <c r="A547" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-01 20:11:45</t>
+        </is>
+      </c>
+      <c r="B547" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C547" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D547" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E547" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F547" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G547" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H547" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I547" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J547" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K547" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="548" ht="20" customHeight="1">
+      <c r="A548" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01 22:14:43</t>
+        </is>
+      </c>
+      <c r="B548" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C548" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E548" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F548" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G548" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H548" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I548" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J548" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K548" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="549" ht="20" customHeight="1">
+      <c r="A549" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-01 22:14:56</t>
+        </is>
+      </c>
+      <c r="B549" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C549" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D549" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E549" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F549" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G549" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H549" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I549" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J549" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K549" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="550" ht="20" customHeight="1">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01 22:47:21</t>
+        </is>
+      </c>
+      <c r="B550" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C550" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E550" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F550" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G550" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H550" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I550" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J550" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K550" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="551" ht="20" customHeight="1">
+      <c r="A551" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02 17:43:14</t>
+        </is>
+      </c>
+      <c r="B551" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C551" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D551" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E551" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F551" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G551" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H551" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I551" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J551" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K551" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="552" ht="20" customHeight="1">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02 17:45:09</t>
+        </is>
+      </c>
+      <c r="B552" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C552" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E552" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F552" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G552" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H552" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I552" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J552" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K552" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="553" ht="20" customHeight="1">
+      <c r="A553" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02 17:57:44</t>
+        </is>
+      </c>
+      <c r="B553" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C553" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D553" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E553" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F553" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G553" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H553" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I553" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J553" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K553" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="554" ht="20" customHeight="1">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02 17:57:48</t>
+        </is>
+      </c>
+      <c r="B554" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C554" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E554" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F554" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G554" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H554" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I554" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J554" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K554" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="555" ht="20" customHeight="1">
+      <c r="A555" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02 18:05:01</t>
+        </is>
+      </c>
+      <c r="B555" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C555" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D555" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E555" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F555" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G555" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H555" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I555" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J555" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K555" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="556" ht="20" customHeight="1">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02 18:05:08</t>
+        </is>
+      </c>
+      <c r="B556" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C556" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E556" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F556" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G556" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H556" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I556" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J556" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K556" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="557" ht="20" customHeight="1">
+      <c r="A557" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-02 18:12:53</t>
+        </is>
+      </c>
+      <c r="B557" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C557" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D557" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E557" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F557" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G557" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H557" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I557" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J557" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K557" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="558" ht="20" customHeight="1">
+      <c r="A558" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02 18:13:01</t>
+        </is>
+      </c>
+      <c r="B558" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C558" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E558" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F558" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G558" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H558" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I558" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J558" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K558" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
style: fix welcome screen logo clipping on desktop overflow and configure local Ollama detection
</commit_message>
<xml_diff>
--- a/api_key_metrics.xlsx
+++ b/api_key_metrics.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K559"/>
+  <dimension ref="A1:K560"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -30171,6 +30171,59 @@
         </is>
       </c>
     </row>
+    <row r="560" ht="20" customHeight="1">
+      <c r="A560" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:17:23</t>
+        </is>
+      </c>
+      <c r="B560" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C560" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D560" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E560" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F560" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G560" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H560" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I560" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J560" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K560" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: collapse consecutive role messages in all API stream functions and update sidecar binaries
</commit_message>
<xml_diff>
--- a/api_key_metrics.xlsx
+++ b/api_key_metrics.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K560"/>
+  <dimension ref="A1:K586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -30224,6 +30224,1384 @@
         </is>
       </c>
     </row>
+    <row r="561" ht="20" customHeight="1">
+      <c r="A561" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:24:25</t>
+        </is>
+      </c>
+      <c r="B561" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C561" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D561" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E561" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F561" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G561" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H561" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I561" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J561" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K561" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="562" ht="20" customHeight="1">
+      <c r="A562" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:24:44</t>
+        </is>
+      </c>
+      <c r="B562" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C562" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D562" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E562" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F562" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G562" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H562" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I562" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J562" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K562" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="563" ht="20" customHeight="1">
+      <c r="A563" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:27:34</t>
+        </is>
+      </c>
+      <c r="B563" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C563" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D563" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E563" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F563" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G563" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H563" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I563" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J563" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K563" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="564" ht="20" customHeight="1">
+      <c r="A564" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:27:43</t>
+        </is>
+      </c>
+      <c r="B564" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C564" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D564" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E564" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F564" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G564" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H564" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I564" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J564" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K564" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="565" ht="20" customHeight="1">
+      <c r="A565" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:32:35</t>
+        </is>
+      </c>
+      <c r="B565" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C565" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D565" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E565" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F565" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G565" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H565" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I565" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J565" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K565" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="566" ht="20" customHeight="1">
+      <c r="A566" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:32:52</t>
+        </is>
+      </c>
+      <c r="B566" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C566" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D566" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E566" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F566" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G566" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H566" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I566" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J566" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K566" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="567" ht="20" customHeight="1">
+      <c r="A567" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:33:02</t>
+        </is>
+      </c>
+      <c r="B567" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C567" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D567" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E567" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F567" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G567" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H567" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I567" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J567" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K567" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="568" ht="20" customHeight="1">
+      <c r="A568" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:33:06</t>
+        </is>
+      </c>
+      <c r="B568" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C568" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D568" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E568" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F568" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G568" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H568" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I568" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J568" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K568" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="569" ht="20" customHeight="1">
+      <c r="A569" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:35:16</t>
+        </is>
+      </c>
+      <c r="B569" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C569" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D569" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E569" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F569" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G569" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H569" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I569" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J569" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K569" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="570" ht="20" customHeight="1">
+      <c r="A570" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:35:24</t>
+        </is>
+      </c>
+      <c r="B570" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C570" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D570" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E570" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F570" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G570" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H570" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I570" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J570" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K570" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="571" ht="20" customHeight="1">
+      <c r="A571" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:03</t>
+        </is>
+      </c>
+      <c r="B571" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C571" s="5" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D571" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E571" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F571" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G571" s="5" t="inlineStr">
+        <is>
+          <t>complex_reasoning</t>
+        </is>
+      </c>
+      <c r="H571" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I571" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J571" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K571" s="6" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="572" ht="20" customHeight="1">
+      <c r="A572" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:35</t>
+        </is>
+      </c>
+      <c r="B572" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C572" s="2" t="inlineStr">
+        <is>
+          <t>QUARANTINE</t>
+        </is>
+      </c>
+      <c r="D572" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E572" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F572" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G572" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H572" s="7" t="inlineStr">
+        <is>
+          <t>QUARANTINED</t>
+        </is>
+      </c>
+      <c r="I572" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J572" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K572" s="3" t="inlineStr">
+        <is>
+          <t>Key quarantined for 5m. Error: cannot access local variable 'uuid' where it is not associated with a value</t>
+        </is>
+      </c>
+    </row>
+    <row r="573" ht="20" customHeight="1">
+      <c r="A573" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:36</t>
+        </is>
+      </c>
+      <c r="B573" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C573" s="5" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D573" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E573" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F573" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G573" s="5" t="inlineStr">
+        <is>
+          <t>complex_reasoning</t>
+        </is>
+      </c>
+      <c r="H573" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I573" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J573" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K573" s="6" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="574" ht="20" customHeight="1">
+      <c r="A574" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:37</t>
+        </is>
+      </c>
+      <c r="B574" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C574" s="2" t="inlineStr">
+        <is>
+          <t>QUARANTINE</t>
+        </is>
+      </c>
+      <c r="D574" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E574" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F574" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G574" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H574" s="7" t="inlineStr">
+        <is>
+          <t>QUARANTINED</t>
+        </is>
+      </c>
+      <c r="I574" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J574" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K574" s="3" t="inlineStr">
+        <is>
+          <t>Key quarantined for 5m. Error: cannot access local variable 'uuid' where it is not associated with a value</t>
+        </is>
+      </c>
+    </row>
+    <row r="575" ht="20" customHeight="1">
+      <c r="A575" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:38</t>
+        </is>
+      </c>
+      <c r="B575" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C575" s="5" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D575" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E575" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F575" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G575" s="5" t="inlineStr">
+        <is>
+          <t>complex_reasoning</t>
+        </is>
+      </c>
+      <c r="H575" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I575" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J575" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K575" s="6" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="576" ht="20" customHeight="1">
+      <c r="A576" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:39</t>
+        </is>
+      </c>
+      <c r="B576" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C576" s="2" t="inlineStr">
+        <is>
+          <t>QUARANTINE</t>
+        </is>
+      </c>
+      <c r="D576" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E576" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F576" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G576" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H576" s="7" t="inlineStr">
+        <is>
+          <t>QUARANTINED</t>
+        </is>
+      </c>
+      <c r="I576" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J576" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K576" s="3" t="inlineStr">
+        <is>
+          <t>Key quarantined for 5m. Error: Ollama Error (400): {"error":"{\"error\":{\"code\":400,\"message\":\"Cannot have 2 or more assistant messages at the end of the list.\",\"type\":\"invalid_request_error\"}}"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="577" ht="20" customHeight="1">
+      <c r="A577" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:40</t>
+        </is>
+      </c>
+      <c r="B577" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C577" s="5" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D577" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E577" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F577" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G577" s="5" t="inlineStr">
+        <is>
+          <t>complex_reasoning</t>
+        </is>
+      </c>
+      <c r="H577" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I577" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J577" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K577" s="6" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="578" ht="20" customHeight="1">
+      <c r="A578" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:41</t>
+        </is>
+      </c>
+      <c r="B578" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C578" s="2" t="inlineStr">
+        <is>
+          <t>QUARANTINE</t>
+        </is>
+      </c>
+      <c r="D578" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E578" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F578" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G578" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H578" s="7" t="inlineStr">
+        <is>
+          <t>QUARANTINED</t>
+        </is>
+      </c>
+      <c r="I578" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J578" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K578" s="3" t="inlineStr">
+        <is>
+          <t>Key quarantined for 5m. Error: Ollama Error (400): {"error":"{\"error\":{\"code\":400,\"message\":\"Cannot have 2 or more assistant messages at the end of the list.\",\"type\":\"invalid_request_error\"}}"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="579" ht="20" customHeight="1">
+      <c r="A579" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:42</t>
+        </is>
+      </c>
+      <c r="B579" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C579" s="5" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D579" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E579" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F579" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G579" s="5" t="inlineStr">
+        <is>
+          <t>complex_reasoning</t>
+        </is>
+      </c>
+      <c r="H579" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I579" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J579" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K579" s="6" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="580" ht="20" customHeight="1">
+      <c r="A580" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:37:43</t>
+        </is>
+      </c>
+      <c r="B580" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C580" s="2" t="inlineStr">
+        <is>
+          <t>QUARANTINE</t>
+        </is>
+      </c>
+      <c r="D580" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E580" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F580" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G580" s="2" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H580" s="7" t="inlineStr">
+        <is>
+          <t>QUARANTINED</t>
+        </is>
+      </c>
+      <c r="I580" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J580" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K580" s="3" t="inlineStr">
+        <is>
+          <t>Key quarantined for 5m. Error: Ollama Error (400): {"error":"{\"error\":{\"code\":400,\"message\":\"Cannot have 2 or more assistant messages at the end of the list.\",\"type\":\"invalid_request_error\"}}"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="581" ht="20" customHeight="1">
+      <c r="A581" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:40:53</t>
+        </is>
+      </c>
+      <c r="B581" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C581" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D581" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E581" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F581" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G581" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H581" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I581" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J581" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K581" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="582" ht="20" customHeight="1">
+      <c r="A582" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:40:58</t>
+        </is>
+      </c>
+      <c r="B582" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C582" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D582" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E582" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F582" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G582" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H582" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I582" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J582" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K582" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="583" ht="20" customHeight="1">
+      <c r="A583" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:41:06</t>
+        </is>
+      </c>
+      <c r="B583" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C583" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D583" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E583" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F583" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G583" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H583" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I583" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J583" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K583" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="584" ht="20" customHeight="1">
+      <c r="A584" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:41:12</t>
+        </is>
+      </c>
+      <c r="B584" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C584" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D584" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E584" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F584" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G584" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H584" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I584" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J584" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K584" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="585" ht="20" customHeight="1">
+      <c r="A585" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:41:19</t>
+        </is>
+      </c>
+      <c r="B585" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C585" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D585" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E585" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F585" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G585" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H585" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I585" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J585" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K585" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="586" ht="20" customHeight="1">
+      <c r="A586" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:41:29</t>
+        </is>
+      </c>
+      <c r="B586" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C586" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D586" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E586" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F586" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G586" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H586" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I586" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J586" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K586" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Render + Desktop_App + T&C
</commit_message>
<xml_diff>
--- a/api_key_metrics.xlsx
+++ b/api_key_metrics.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K586"/>
+  <dimension ref="A1:K603"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -31602,6 +31602,907 @@
         </is>
       </c>
     </row>
+    <row r="587" ht="20" customHeight="1">
+      <c r="A587" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:48:22</t>
+        </is>
+      </c>
+      <c r="B587" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C587" s="5" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D587" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E587" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F587" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G587" s="5" t="inlineStr">
+        <is>
+          <t>complex_reasoning</t>
+        </is>
+      </c>
+      <c r="H587" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I587" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J587" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K587" s="6" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="588" ht="20" customHeight="1">
+      <c r="A588" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:48:37</t>
+        </is>
+      </c>
+      <c r="B588" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C588" s="2" t="inlineStr">
+        <is>
+          <t>EXECUTE</t>
+        </is>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E588" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F588" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G588" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H588" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I588" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="J588" s="2" t="n">
+        <v>15.413</v>
+      </c>
+      <c r="K588" s="3" t="inlineStr">
+        <is>
+          <t>Successful request execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="589" ht="20" customHeight="1">
+      <c r="A589" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 17:07:48</t>
+        </is>
+      </c>
+      <c r="B589" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C589" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D589" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E589" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F589" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G589" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H589" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I589" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J589" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K589" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="590" ht="20" customHeight="1">
+      <c r="A590" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 18:01:08</t>
+        </is>
+      </c>
+      <c r="B590" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C590" s="2" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D590" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E590" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F590" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G590" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H590" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I590" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J590" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K590" s="3" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="591" ht="20" customHeight="1">
+      <c r="A591" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 18:01:46</t>
+        </is>
+      </c>
+      <c r="B591" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C591" s="5" t="inlineStr">
+        <is>
+          <t>EXECUTE</t>
+        </is>
+      </c>
+      <c r="D591" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E591" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F591" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G591" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H591" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I591" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="J591" s="5" t="n">
+        <v>35.204</v>
+      </c>
+      <c r="K591" s="6" t="inlineStr">
+        <is>
+          <t>Successful request execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="592" ht="20" customHeight="1">
+      <c r="A592" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 18:02:25</t>
+        </is>
+      </c>
+      <c r="B592" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C592" s="2" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D592" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E592" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F592" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G592" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H592" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I592" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J592" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K592" s="3" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="593" ht="20" customHeight="1">
+      <c r="A593" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 18:02:38</t>
+        </is>
+      </c>
+      <c r="B593" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C593" s="5" t="inlineStr">
+        <is>
+          <t>EXECUTE</t>
+        </is>
+      </c>
+      <c r="D593" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E593" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F593" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G593" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H593" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I593" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="J593" s="5" t="n">
+        <v>11.378</v>
+      </c>
+      <c r="K593" s="6" t="inlineStr">
+        <is>
+          <t>Successful request execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="594" ht="20" customHeight="1">
+      <c r="A594" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 18:03:03</t>
+        </is>
+      </c>
+      <c r="B594" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C594" s="2" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E594" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F594" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G594" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H594" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I594" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J594" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K594" s="3" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="595" ht="20" customHeight="1">
+      <c r="A595" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 18:03:13</t>
+        </is>
+      </c>
+      <c r="B595" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C595" s="5" t="inlineStr">
+        <is>
+          <t>EXECUTE</t>
+        </is>
+      </c>
+      <c r="D595" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E595" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F595" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G595" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H595" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I595" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="J595" s="5" t="n">
+        <v>8.972</v>
+      </c>
+      <c r="K595" s="6" t="inlineStr">
+        <is>
+          <t>Successful request execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="596" ht="20" customHeight="1">
+      <c r="A596" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 18:03:39</t>
+        </is>
+      </c>
+      <c r="B596" s="3" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C596" s="2" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="D596" s="2" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E596" s="3" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F596" s="3" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G596" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H596" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I596" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J596" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K596" s="3" t="inlineStr">
+        <is>
+          <t>Routed optimally by KeyOptimus</t>
+        </is>
+      </c>
+    </row>
+    <row r="597" ht="20" customHeight="1">
+      <c r="A597" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 18:03:53</t>
+        </is>
+      </c>
+      <c r="B597" s="6" t="inlineStr">
+        <is>
+          <t>single_session</t>
+        </is>
+      </c>
+      <c r="C597" s="5" t="inlineStr">
+        <is>
+          <t>EXECUTE</t>
+        </is>
+      </c>
+      <c r="D597" s="5" t="inlineStr">
+        <is>
+          <t>ollama</t>
+        </is>
+      </c>
+      <c r="E597" s="6" t="inlineStr">
+        <is>
+          <t>Local Ollama Engine</t>
+        </is>
+      </c>
+      <c r="F597" s="6" t="inlineStr">
+        <is>
+          <t>devops-concierge-coder:latest</t>
+        </is>
+      </c>
+      <c r="G597" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H597" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I597" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="J597" s="5" t="n">
+        <v>12.455</v>
+      </c>
+      <c r="K597" s="6" t="inlineStr">
+        <is>
+          <t>Successful request execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="598" ht="20" customHeight="1">
+      <c r="A598" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 19:11:03</t>
+        </is>
+      </c>
+      <c r="B598" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C598" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D598" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E598" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F598" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G598" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H598" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I598" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J598" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K598" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="599" ht="20" customHeight="1">
+      <c r="A599" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 19:14:17</t>
+        </is>
+      </c>
+      <c r="B599" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C599" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D599" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E599" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F599" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G599" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H599" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I599" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J599" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K599" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="600" ht="20" customHeight="1">
+      <c r="A600" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 19:14:22</t>
+        </is>
+      </c>
+      <c r="B600" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C600" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D600" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E600" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F600" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G600" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H600" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I600" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J600" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K600" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="601" ht="20" customHeight="1">
+      <c r="A601" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 19:14:29</t>
+        </is>
+      </c>
+      <c r="B601" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C601" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D601" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E601" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F601" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G601" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H601" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I601" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J601" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K601" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="602" ht="20" customHeight="1">
+      <c r="A602" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 19:30:07</t>
+        </is>
+      </c>
+      <c r="B602" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C602" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D602" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E602" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F602" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G602" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H602" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I602" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J602" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K602" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
+    <row r="603" ht="20" customHeight="1">
+      <c r="A603" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03 19:36:54</t>
+        </is>
+      </c>
+      <c r="B603" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C603" s="5" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D603" s="5" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E603" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F603" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G603" s="5" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H603" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I603" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J603" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K603" s="6" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Show live app URL and dashboard URL on deployment success
</commit_message>
<xml_diff>
--- a/api_key_metrics.xlsx
+++ b/api_key_metrics.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K603"/>
+  <dimension ref="A1:K604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -32503,6 +32503,59 @@
         </is>
       </c>
     </row>
+    <row r="604" ht="20" customHeight="1">
+      <c r="A604" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03 19:42:30</t>
+        </is>
+      </c>
+      <c r="B604" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="C604" s="2" t="inlineStr">
+        <is>
+          <t>STARTUP</t>
+        </is>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="E604" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="F604" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G604" s="2" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="H604" s="4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="I604" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J604" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K604" s="3" t="inlineStr">
+        <is>
+          <t>KeyOptimus microservice successfully initialized and running on port 8005</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>